<commit_message>
Load state-league history (VFL/WAFL/SANFL) for 2021-2025 vfl_only flags.
Scrape and cache VFL+WAFL from 2021 and SANFL where PDFs exist; rebuild availability so reserves weeks are marked vfl_only instead of unavailable.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/shared/output/exports/collingwood_2021_deep_dive.xlsx
+++ b/shared/output/exports/collingwood_2021_deep_dive.xlsx
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>931.4</v>
+        <v>803.2</v>
       </c>
     </row>
     <row r="7">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>915</v>
+        <v>793.9</v>
       </c>
     </row>
     <row r="8">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.3</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -581,55 +581,60 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>rank_delta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>player_rounds_lost</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>players_with_absences</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>games_missed_slots</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>pvs_games_missed</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>pvs_all_absences</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>pvs_vfl_only</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pvs_top5_round_sum</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>rank_games_missed_pvs</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>rank_all_absence_pvs</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>rank_top5_sum</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rank_slots_lost</t>
         </is>
@@ -648,28 +653,28 @@
         <v>5</v>
       </c>
       <c r="D2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="E2" t="n">
         <v>396</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>37</v>
       </c>
-      <c r="F2" t="n">
-        <v>396</v>
-      </c>
       <c r="G2" t="n">
+        <v>321</v>
+      </c>
+      <c r="H2" t="n">
+        <v>983.1</v>
+      </c>
+      <c r="I2" t="n">
         <v>1174.9</v>
       </c>
-      <c r="H2" t="n">
-        <v>1174.9</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
       <c r="J2" t="n">
+        <v>191.8</v>
+      </c>
+      <c r="K2" t="n">
         <v>507.3</v>
-      </c>
-      <c r="K2" t="n">
-        <v>18</v>
       </c>
       <c r="L2" t="n">
         <v>18</v>
@@ -680,6 +685,9 @@
       <c r="N2" t="n">
         <v>18</v>
       </c>
+      <c r="O2" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -694,129 +702,138 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
+        <v>-7</v>
+      </c>
+      <c r="E3" t="n">
         <v>352</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>35</v>
       </c>
-      <c r="F3" t="n">
-        <v>352</v>
-      </c>
       <c r="G3" t="n">
+        <v>310</v>
+      </c>
+      <c r="H3" t="n">
+        <v>971.1</v>
+      </c>
+      <c r="I3" t="n">
         <v>1080.8</v>
       </c>
-      <c r="H3" t="n">
-        <v>1080.8</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
       <c r="J3" t="n">
+        <v>109.6</v>
+      </c>
+      <c r="K3" t="n">
         <v>456.6</v>
-      </c>
-      <c r="K3" t="n">
-        <v>17</v>
       </c>
       <c r="L3" t="n">
         <v>17</v>
       </c>
       <c r="M3" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="N3" t="n">
         <v>12</v>
       </c>
+      <c r="O3" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Gold Coast</t>
+          <t>Carlton</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>330</v>
+        <v>-3</v>
       </c>
       <c r="E4" t="n">
+        <v>352</v>
+      </c>
+      <c r="F4" t="n">
         <v>35</v>
       </c>
-      <c r="F4" t="n">
-        <v>330</v>
-      </c>
       <c r="G4" t="n">
-        <v>1059</v>
+        <v>308</v>
       </c>
       <c r="H4" t="n">
-        <v>1059</v>
+        <v>907.8</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1012.5</v>
       </c>
       <c r="J4" t="n">
-        <v>481</v>
+        <v>104.7</v>
       </c>
       <c r="K4" t="n">
-        <v>16</v>
+        <v>429.9</v>
       </c>
       <c r="L4" t="n">
         <v>16</v>
       </c>
       <c r="M4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N4" t="n">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="O4" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Carlton</t>
+          <t>North Melbourne</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>352</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>35</v>
+        <v>330</v>
       </c>
       <c r="F5" t="n">
-        <v>352</v>
+        <v>33</v>
       </c>
       <c r="G5" t="n">
-        <v>1012.5</v>
+        <v>295</v>
       </c>
       <c r="H5" t="n">
-        <v>1012.5</v>
+        <v>898.4</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>977.8</v>
       </c>
       <c r="J5" t="n">
-        <v>429.9</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>15</v>
+        <v>485.8</v>
       </c>
       <c r="L5" t="n">
         <v>15</v>
       </c>
       <c r="M5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N5" t="n">
-        <v>12</v>
+        <v>17</v>
+      </c>
+      <c r="O5" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -832,313 +849,334 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
+        <v>-7</v>
+      </c>
+      <c r="E6" t="n">
         <v>308</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>33</v>
       </c>
-      <c r="F6" t="n">
-        <v>308</v>
-      </c>
       <c r="G6" t="n">
+        <v>268</v>
+      </c>
+      <c r="H6" t="n">
+        <v>896.3</v>
+      </c>
+      <c r="I6" t="n">
         <v>1006.1</v>
       </c>
-      <c r="H6" t="n">
-        <v>1006.1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
       <c r="J6" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="K6" t="n">
         <v>466.8</v>
-      </c>
-      <c r="K6" t="n">
-        <v>14</v>
       </c>
       <c r="L6" t="n">
         <v>14</v>
       </c>
       <c r="M6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N6" t="n">
         <v>15</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fremantle</t>
+          <t>Gold Coast</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>352</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
+        <v>330</v>
+      </c>
+      <c r="F7" t="n">
         <v>35</v>
       </c>
-      <c r="F7" t="n">
-        <v>352</v>
-      </c>
       <c r="G7" t="n">
-        <v>1005.8</v>
+        <v>260</v>
       </c>
       <c r="H7" t="n">
-        <v>1005.8</v>
+        <v>852.5</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1059</v>
       </c>
       <c r="J7" t="n">
-        <v>415.8</v>
+        <v>206.5</v>
       </c>
       <c r="K7" t="n">
-        <v>13</v>
+        <v>481</v>
       </c>
       <c r="L7" t="n">
         <v>13</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="N7" t="n">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="O7" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Greater Western Sydney</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>374</v>
+        <v>-4</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>352</v>
       </c>
       <c r="F8" t="n">
-        <v>374</v>
+        <v>35</v>
       </c>
       <c r="G8" t="n">
-        <v>994.6</v>
+        <v>310</v>
       </c>
       <c r="H8" t="n">
-        <v>994.6</v>
+        <v>845.7</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>938.2</v>
       </c>
       <c r="J8" t="n">
-        <v>466</v>
+        <v>92.5</v>
       </c>
       <c r="K8" t="n">
-        <v>12</v>
+        <v>428</v>
       </c>
       <c r="L8" t="n">
         <v>12</v>
       </c>
       <c r="M8" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="N8" t="n">
-        <v>17</v>
+        <v>7</v>
+      </c>
+      <c r="O8" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>North Melbourne</t>
+          <t>Hawthorn</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
         <v>330</v>
       </c>
-      <c r="E9" t="n">
-        <v>33</v>
-      </c>
       <c r="F9" t="n">
-        <v>330</v>
+        <v>34</v>
       </c>
       <c r="G9" t="n">
-        <v>977.8</v>
+        <v>275</v>
       </c>
       <c r="H9" t="n">
-        <v>977.8</v>
+        <v>839.4</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>962.2</v>
       </c>
       <c r="J9" t="n">
-        <v>485.8</v>
+        <v>122.8</v>
       </c>
       <c r="K9" t="n">
-        <v>11</v>
+        <v>453.6</v>
       </c>
       <c r="L9" t="n">
         <v>11</v>
       </c>
       <c r="M9" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="N9" t="n">
+        <v>11</v>
+      </c>
+      <c r="O9" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hawthorn</t>
+          <t>Port Adelaide</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>330</v>
+        <v>-8</v>
       </c>
       <c r="E10" t="n">
-        <v>34</v>
+        <v>264</v>
       </c>
       <c r="F10" t="n">
-        <v>330</v>
+        <v>27</v>
       </c>
       <c r="G10" t="n">
-        <v>962.2</v>
+        <v>264</v>
       </c>
       <c r="H10" t="n">
-        <v>962.2</v>
+        <v>830.2</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>830.2</v>
       </c>
       <c r="J10" t="n">
-        <v>453.6</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>10</v>
+        <v>460.3</v>
       </c>
       <c r="L10" t="n">
         <v>10</v>
       </c>
       <c r="M10" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N10" t="n">
-        <v>9</v>
+        <v>13</v>
+      </c>
+      <c r="O10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Greater Western Sydney</t>
+          <t>Fremantle</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="n">
         <v>11</v>
       </c>
-      <c r="C11" t="n">
-        <v>8</v>
-      </c>
       <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
         <v>352</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>35</v>
       </c>
-      <c r="F11" t="n">
-        <v>352</v>
-      </c>
       <c r="G11" t="n">
-        <v>938.2</v>
+        <v>281</v>
       </c>
       <c r="H11" t="n">
-        <v>938.2</v>
+        <v>825.9</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1005.8</v>
       </c>
       <c r="J11" t="n">
-        <v>428</v>
+        <v>180</v>
       </c>
       <c r="K11" t="n">
-        <v>9</v>
+        <v>415.8</v>
       </c>
       <c r="L11" t="n">
         <v>9</v>
       </c>
       <c r="M11" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="N11" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D12" t="n">
-        <v>308</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>33</v>
+        <v>374</v>
       </c>
       <c r="F12" t="n">
-        <v>308</v>
+        <v>36</v>
       </c>
       <c r="G12" t="n">
-        <v>933.7</v>
+        <v>288</v>
       </c>
       <c r="H12" t="n">
-        <v>933.7</v>
+        <v>820</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>994.6</v>
       </c>
       <c r="J12" t="n">
-        <v>442.4</v>
+        <v>174.6</v>
       </c>
       <c r="K12" t="n">
-        <v>8</v>
+        <v>466</v>
       </c>
       <c r="L12" t="n">
         <v>8</v>
       </c>
       <c r="M12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>14</v>
+      </c>
+      <c r="O12" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -1154,129 +1192,138 @@
         <v>17</v>
       </c>
       <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="n">
         <v>352</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>36</v>
       </c>
-      <c r="F13" t="n">
-        <v>352</v>
-      </c>
       <c r="G13" t="n">
+        <v>290</v>
+      </c>
+      <c r="H13" t="n">
+        <v>803.2</v>
+      </c>
+      <c r="I13" t="n">
         <v>931.4</v>
       </c>
-      <c r="H13" t="n">
-        <v>931.4</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
       <c r="J13" t="n">
+        <v>128.2</v>
+      </c>
+      <c r="K13" t="n">
         <v>416.2</v>
-      </c>
-      <c r="K13" t="n">
-        <v>7</v>
       </c>
       <c r="L13" t="n">
         <v>7</v>
       </c>
       <c r="M13" t="n">
+        <v>7</v>
+      </c>
+      <c r="N13" t="n">
         <v>5</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>West Coast</t>
+          <t>Adelaide</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" t="n">
         <v>9</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>308</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>32</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>308</v>
       </c>
-      <c r="G14" t="n">
-        <v>841.6</v>
-      </c>
       <c r="H14" t="n">
-        <v>841.6</v>
+        <v>785.1</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>785.1</v>
       </c>
       <c r="J14" t="n">
-        <v>427.9</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>6</v>
+        <v>408.3</v>
       </c>
       <c r="L14" t="n">
         <v>6</v>
       </c>
       <c r="M14" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N14" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Port Adelaide</t>
+          <t>Sydney</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>264</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>27</v>
+        <v>308</v>
       </c>
       <c r="F15" t="n">
-        <v>264</v>
+        <v>33</v>
       </c>
       <c r="G15" t="n">
-        <v>830.2</v>
+        <v>249</v>
       </c>
       <c r="H15" t="n">
-        <v>830.2</v>
+        <v>769.7</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>933.7</v>
       </c>
       <c r="J15" t="n">
-        <v>460.3</v>
+        <v>164</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>442.4</v>
       </c>
       <c r="L15" t="n">
         <v>5</v>
       </c>
       <c r="M15" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N15" t="n">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="O15" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -1292,82 +1339,88 @@
         <v>3</v>
       </c>
       <c r="D16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E16" t="n">
         <v>264</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>33</v>
       </c>
-      <c r="F16" t="n">
-        <v>264</v>
-      </c>
       <c r="G16" t="n">
+        <v>227</v>
+      </c>
+      <c r="H16" t="n">
+        <v>696</v>
+      </c>
+      <c r="I16" t="n">
         <v>788</v>
       </c>
-      <c r="H16" t="n">
-        <v>788</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
       <c r="J16" t="n">
+        <v>92</v>
+      </c>
+      <c r="K16" t="n">
         <v>439.5</v>
-      </c>
-      <c r="K16" t="n">
-        <v>4</v>
       </c>
       <c r="L16" t="n">
         <v>4</v>
       </c>
       <c r="M16" t="n">
+        <v>4</v>
+      </c>
+      <c r="N16" t="n">
         <v>9</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Adelaide</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="n">
         <v>308</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>32</v>
       </c>
-      <c r="F17" t="n">
-        <v>308</v>
-      </c>
       <c r="G17" t="n">
-        <v>785.1</v>
+        <v>204</v>
       </c>
       <c r="H17" t="n">
-        <v>785.1</v>
+        <v>600.3</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>841.6</v>
       </c>
       <c r="J17" t="n">
-        <v>408.3</v>
+        <v>241.3</v>
       </c>
       <c r="K17" t="n">
-        <v>3</v>
+        <v>427.9</v>
       </c>
       <c r="L17" t="n">
         <v>3</v>
       </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1384,36 +1437,39 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E18" t="n">
         <v>242</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>24</v>
       </c>
-      <c r="F18" t="n">
-        <v>242</v>
-      </c>
       <c r="G18" t="n">
+        <v>197</v>
+      </c>
+      <c r="H18" t="n">
+        <v>548.4</v>
+      </c>
+      <c r="I18" t="n">
         <v>668.3</v>
       </c>
-      <c r="H18" t="n">
-        <v>668.3</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
       <c r="J18" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="K18" t="n">
         <v>411.1</v>
-      </c>
-      <c r="K18" t="n">
-        <v>2</v>
       </c>
       <c r="L18" t="n">
         <v>2</v>
       </c>
       <c r="M18" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" t="n">
         <v>3</v>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1430,28 +1486,28 @@
         <v>4</v>
       </c>
       <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
         <v>198</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>24</v>
       </c>
-      <c r="F19" t="n">
-        <v>198</v>
-      </c>
       <c r="G19" t="n">
+        <v>166</v>
+      </c>
+      <c r="H19" t="n">
+        <v>416.9</v>
+      </c>
+      <c r="I19" t="n">
         <v>480.7</v>
       </c>
-      <c r="H19" t="n">
-        <v>480.7</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
       <c r="J19" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="K19" t="n">
         <v>352.8</v>
-      </c>
-      <c r="K19" t="n">
-        <v>1</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1460,6 +1516,9 @@
         <v>1</v>
       </c>
       <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3799,13 +3858,13 @@
         <v>4</v>
       </c>
       <c r="M19" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O19" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P19" t="n">
         <v>3.059</v>
@@ -3832,7 +3891,7 @@
         <v>3.4535</v>
       </c>
       <c r="X19" t="n">
-        <v>55.1</v>
+        <v>42.8</v>
       </c>
       <c r="Y19" t="n">
         <v>0</v>
@@ -3922,13 +3981,13 @@
         <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O20" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="P20" t="n">
         <v>2.982</v>
@@ -3955,7 +4014,7 @@
         <v>3.3669</v>
       </c>
       <c r="X20" t="n">
-        <v>59.6</v>
+        <v>44.7</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -4294,10 +4353,10 @@
         <v>7</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P23" t="n">
         <v>2.85</v>
@@ -4324,7 +4383,7 @@
         <v>3.2178</v>
       </c>
       <c r="X23" t="n">
-        <v>31.4</v>
+        <v>25.7</v>
       </c>
       <c r="Y23" t="n">
         <v>0.182</v>
@@ -4660,13 +4719,13 @@
         <v>7</v>
       </c>
       <c r="M26" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P26" t="n">
         <v>2.452</v>
@@ -4693,7 +4752,7 @@
         <v>2.769</v>
       </c>
       <c r="X26" t="n">
-        <v>36.8</v>
+        <v>31.9</v>
       </c>
       <c r="Y26" t="n">
         <v>0.143</v>
@@ -4783,13 +4842,13 @@
         <v>7</v>
       </c>
       <c r="M27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P27" t="n">
         <v>2.443</v>
@@ -4816,7 +4875,7 @@
         <v>2.759</v>
       </c>
       <c r="X27" t="n">
-        <v>40.7</v>
+        <v>35.3</v>
       </c>
       <c r="Y27" t="n">
         <v>1.143</v>
@@ -4909,10 +4968,10 @@
         <v>10</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P28" t="n">
         <v>2.38</v>
@@ -4939,7 +4998,7 @@
         <v>2.6876</v>
       </c>
       <c r="X28" t="n">
-        <v>23.8</v>
+        <v>19</v>
       </c>
       <c r="Y28" t="n">
         <v>0.583</v>
@@ -5032,10 +5091,10 @@
         <v>9</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O29" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P29" t="n">
         <v>2.355</v>
@@ -5062,7 +5121,7 @@
         <v>2.6596</v>
       </c>
       <c r="X29" t="n">
-        <v>30.6</v>
+        <v>25.9</v>
       </c>
       <c r="Y29" t="n">
         <v>0.111</v>
@@ -5275,13 +5334,13 @@
         <v>9</v>
       </c>
       <c r="M31" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N31" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O31" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P31" t="n">
         <v>2.292</v>
@@ -5308,7 +5367,7 @@
         <v>2.5881</v>
       </c>
       <c r="X31" t="n">
-        <v>29.8</v>
+        <v>20.6</v>
       </c>
       <c r="Y31" t="n">
         <v>0.222</v>
@@ -5398,13 +5457,13 @@
         <v>10</v>
       </c>
       <c r="M32" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N32" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O32" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P32" t="n">
         <v>2.196</v>
@@ -5431,7 +5490,7 @@
         <v>2.3987</v>
       </c>
       <c r="X32" t="n">
-        <v>26.4</v>
+        <v>17.6</v>
       </c>
       <c r="Y32" t="n">
         <v>0.7</v>
@@ -5521,13 +5580,13 @@
         <v>4</v>
       </c>
       <c r="M33" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O33" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="P33" t="n">
         <v>2.185</v>
@@ -5554,7 +5613,7 @@
         <v>2.4665</v>
       </c>
       <c r="X33" t="n">
-        <v>39.3</v>
+        <v>24</v>
       </c>
       <c r="Y33" t="n">
         <v>0</v>
@@ -5647,10 +5706,10 @@
         <v>17</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O34" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="P34" t="n">
         <v>2.051</v>
@@ -5677,7 +5736,7 @@
         <v>2.3162</v>
       </c>
       <c r="X34" t="n">
-        <v>34.9</v>
+        <v>18.5</v>
       </c>
       <c r="Y34" t="n">
         <v>1.2</v>
@@ -5893,10 +5952,10 @@
         <v>5</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P36" t="n">
         <v>1.855</v>
@@ -5923,7 +5982,7 @@
         <v>2.0944</v>
       </c>
       <c r="X36" t="n">
-        <v>13</v>
+        <v>11.1</v>
       </c>
       <c r="Y36" t="n">
         <v>0.067</v>
@@ -6016,10 +6075,10 @@
         <v>21</v>
       </c>
       <c r="N37" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O37" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="P37" t="n">
         <v>1.687</v>
@@ -6046,7 +6105,7 @@
         <v>1.9044</v>
       </c>
       <c r="X37" t="n">
-        <v>35.4</v>
+        <v>21.9</v>
       </c>
       <c r="Y37" t="n">
         <v>0</v>
@@ -6262,10 +6321,10 @@
         <v>12</v>
       </c>
       <c r="N39" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O39" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="P39" t="n">
         <v>1.203</v>
@@ -6292,7 +6351,7 @@
         <v>1.3587</v>
       </c>
       <c r="X39" t="n">
-        <v>20.5</v>
+        <v>15.6</v>
       </c>
       <c r="Y39" t="n">
         <v>0</v>
@@ -6385,10 +6444,10 @@
         <v>20</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O40" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="P40" t="n">
         <v>0.822</v>
@@ -6415,7 +6474,7 @@
         <v>0.7209</v>
       </c>
       <c r="X40" t="n">
-        <v>16.4</v>
+        <v>10.7</v>
       </c>
       <c r="Y40" t="n">
         <v>0</v>
@@ -6572,91 +6631,91 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Max Lynch</t>
+          <t>Jeremy Howe</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ruck</t>
+          <t>key_defender</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.982</v>
+        <v>3.733</v>
       </c>
       <c r="D3" t="n">
-        <v>2.982</v>
+        <v>3.733</v>
       </c>
       <c r="E3" t="n">
-        <v>2.982</v>
+        <v>3.916</v>
       </c>
       <c r="F3" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H3" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>59.6</v>
+        <v>54.8</v>
       </c>
       <c r="L3" t="n">
-        <v>59.6</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mark Keane</t>
+          <t>Max Lynch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>key_defender</t>
+          <t>ruck</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.059</v>
+        <v>2.982</v>
       </c>
       <c r="D4" t="n">
-        <v>3.059</v>
+        <v>2.982</v>
       </c>
       <c r="E4" t="n">
-        <v>3.059</v>
+        <v>2.982</v>
       </c>
       <c r="F4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K4" t="n">
-        <v>55.1</v>
+        <v>44.7</v>
       </c>
       <c r="L4" t="n">
-        <v>55.1</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jeremy Howe</t>
+          <t>Mark Keane</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6665,34 +6724,34 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3.733</v>
+        <v>3.059</v>
       </c>
       <c r="D5" t="n">
-        <v>3.733</v>
+        <v>3.059</v>
       </c>
       <c r="E5" t="n">
-        <v>3.916</v>
+        <v>3.059</v>
       </c>
       <c r="F5" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
         <v>4</v>
       </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
       <c r="K5" t="n">
-        <v>54.8</v>
+        <v>42.8</v>
       </c>
       <c r="L5" t="n">
-        <v>54.8</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="6">
@@ -6740,22 +6799,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mason Cox</t>
+          <t>Tyler Brown</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ruck</t>
+          <t>inside_mid</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.443</v>
+        <v>2.712</v>
       </c>
       <c r="D7" t="n">
-        <v>2.443</v>
+        <v>2.712</v>
       </c>
       <c r="E7" t="n">
-        <v>2.716</v>
+        <v>2.712</v>
       </c>
       <c r="F7" t="n">
         <v>15</v>
@@ -6782,106 +6841,106 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tyler Brown</t>
+          <t>Darcy Moore</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>inside_mid</t>
+          <t>key_defender</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.712</v>
+        <v>4.205</v>
       </c>
       <c r="D8" t="n">
-        <v>2.712</v>
+        <v>4.205</v>
       </c>
       <c r="E8" t="n">
-        <v>2.712</v>
+        <v>4.205</v>
       </c>
       <c r="F8" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G8" t="n">
+        <v>13</v>
+      </c>
+      <c r="H8" t="n">
         <v>7</v>
       </c>
-      <c r="H8" t="n">
-        <v>9</v>
-      </c>
       <c r="I8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>40.7</v>
+        <v>37.8</v>
       </c>
       <c r="L8" t="n">
-        <v>40.7</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tom Wilson</t>
+          <t>Mason Cox</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>utility</t>
+          <t>ruck</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.185</v>
+        <v>2.443</v>
       </c>
       <c r="D9" t="n">
-        <v>2.185</v>
+        <v>2.443</v>
       </c>
       <c r="E9" t="n">
-        <v>2.185</v>
+        <v>2.716</v>
       </c>
       <c r="F9" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H9" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
         <v>2</v>
       </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
       <c r="K9" t="n">
-        <v>39.3</v>
+        <v>35.3</v>
       </c>
       <c r="L9" t="n">
-        <v>39.3</v>
+        <v>40.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Darcy Moore</t>
+          <t>Jamie Elliott</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>key_defender</t>
+          <t>key_forward</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4.205</v>
+        <v>3.602</v>
       </c>
       <c r="D10" t="n">
-        <v>4.205</v>
+        <v>3.602</v>
       </c>
       <c r="E10" t="n">
-        <v>4.205</v>
+        <v>3.602</v>
       </c>
       <c r="F10" t="n">
         <v>9</v>
@@ -6890,19 +6949,19 @@
         <v>13</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>37.8</v>
+        <v>32.4</v>
       </c>
       <c r="L10" t="n">
-        <v>37.8</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="11">
@@ -6932,16 +6991,16 @@
         <v>7</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>36.8</v>
+        <v>31.9</v>
       </c>
       <c r="L11" t="n">
         <v>36.8</v>
@@ -6950,7 +7009,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Anton Tohill</t>
+          <t>Chris Mayne</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6959,40 +7018,40 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.687</v>
+        <v>5.171</v>
       </c>
       <c r="D12" t="n">
-        <v>1.687</v>
+        <v>5.171</v>
       </c>
       <c r="E12" t="n">
-        <v>1.687</v>
+        <v>5.171</v>
       </c>
       <c r="F12" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="H12" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>35.4</v>
+        <v>25.9</v>
       </c>
       <c r="L12" t="n">
-        <v>35.4</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jack Ginnivan</t>
+          <t>Finlay Macrae</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7001,160 +7060,160 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.051</v>
+        <v>2.355</v>
       </c>
       <c r="D13" t="n">
-        <v>2.051</v>
+        <v>2.355</v>
       </c>
       <c r="E13" t="n">
-        <v>2.051</v>
+        <v>2.355</v>
       </c>
       <c r="F13" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G13" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H13" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>34.9</v>
+        <v>25.9</v>
       </c>
       <c r="L13" t="n">
-        <v>34.9</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jamie Elliott</t>
+          <t>Caleb Poulter</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>key_forward</t>
+          <t>inside_mid</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.602</v>
+        <v>2.85</v>
       </c>
       <c r="D14" t="n">
-        <v>3.602</v>
+        <v>2.85</v>
       </c>
       <c r="E14" t="n">
-        <v>3.602</v>
+        <v>2.85</v>
       </c>
       <c r="F14" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G14" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
-        <v>32.4</v>
+        <v>25.7</v>
       </c>
       <c r="L14" t="n">
-        <v>32.4</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Caleb Poulter</t>
+          <t>Tom Wilson</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>inside_mid</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.85</v>
+        <v>2.185</v>
       </c>
       <c r="D15" t="n">
-        <v>2.85</v>
+        <v>2.185</v>
       </c>
       <c r="E15" t="n">
-        <v>2.85</v>
+        <v>2.185</v>
       </c>
       <c r="F15" t="n">
+        <v>18</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" t="n">
         <v>11</v>
       </c>
-      <c r="G15" t="n">
-        <v>11</v>
-      </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
         <v>7</v>
       </c>
-      <c r="I15" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
       <c r="K15" t="n">
-        <v>31.4</v>
+        <v>24</v>
       </c>
       <c r="L15" t="n">
-        <v>31.4</v>
+        <v>39.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Finlay Macrae</t>
+          <t>Anton Tohill</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>utility</t>
+          <t>outside_mid</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.355</v>
+        <v>1.687</v>
       </c>
       <c r="D16" t="n">
-        <v>2.355</v>
+        <v>1.687</v>
       </c>
       <c r="E16" t="n">
-        <v>2.355</v>
+        <v>1.687</v>
       </c>
       <c r="F16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
         <v>13</v>
       </c>
-      <c r="G16" t="n">
-        <v>9</v>
-      </c>
-      <c r="H16" t="n">
-        <v>9</v>
-      </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K16" t="n">
-        <v>30.6</v>
+        <v>21.9</v>
       </c>
       <c r="L16" t="n">
-        <v>30.6</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="17">
@@ -7184,16 +7243,16 @@
         <v>9</v>
       </c>
       <c r="H17" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" t="n">
         <v>4</v>
       </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
       <c r="K17" t="n">
-        <v>29.8</v>
+        <v>20.6</v>
       </c>
       <c r="L17" t="n">
         <v>29.8</v>
@@ -7202,31 +7261,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Oliver Henry</t>
+          <t>Scott Pendlebury</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>utility</t>
+          <t>inside_mid</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.196</v>
+        <v>4.831</v>
       </c>
       <c r="D18" t="n">
-        <v>2.124</v>
+        <v>4.831</v>
       </c>
       <c r="E18" t="n">
-        <v>2.196</v>
+        <v>4.831</v>
       </c>
       <c r="F18" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G18" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="H18" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
         <v>3</v>
@@ -7235,58 +7294,58 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>26.4</v>
+        <v>19.3</v>
       </c>
       <c r="L18" t="n">
-        <v>26.4</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Chris Mayne</t>
+          <t>Trent Bianco</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>outside_mid</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.171</v>
+        <v>2.38</v>
       </c>
       <c r="D19" t="n">
-        <v>5.171</v>
+        <v>2.38</v>
       </c>
       <c r="E19" t="n">
-        <v>5.171</v>
+        <v>2.38</v>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G19" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H19" t="n">
+        <v>8</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
         <v>2</v>
       </c>
-      <c r="I19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
       <c r="K19" t="n">
-        <v>25.9</v>
+        <v>19</v>
       </c>
       <c r="L19" t="n">
-        <v>25.9</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trent Bianco</t>
+          <t>Jack Ginnivan</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7295,40 +7354,40 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.38</v>
+        <v>2.051</v>
       </c>
       <c r="D20" t="n">
-        <v>2.38</v>
+        <v>2.051</v>
       </c>
       <c r="E20" t="n">
-        <v>2.38</v>
+        <v>2.051</v>
       </c>
       <c r="F20" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G20" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K20" t="n">
-        <v>23.8</v>
+        <v>18.5</v>
       </c>
       <c r="L20" t="n">
-        <v>23.8</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jay Rantall</t>
+          <t>Josh Daicos</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7337,82 +7396,82 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.203</v>
+        <v>3.565</v>
       </c>
       <c r="D21" t="n">
-        <v>1.203</v>
+        <v>3.565</v>
       </c>
       <c r="E21" t="n">
-        <v>1.203</v>
+        <v>3.565</v>
       </c>
       <c r="F21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="n">
         <v>17</v>
       </c>
-      <c r="G21" t="n">
-        <v>5</v>
-      </c>
       <c r="H21" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>20.5</v>
+        <v>17.8</v>
       </c>
       <c r="L21" t="n">
-        <v>20.5</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Scott Pendlebury</t>
+          <t>Oliver Henry</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>inside_mid</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4.831</v>
+        <v>2.196</v>
       </c>
       <c r="D22" t="n">
-        <v>4.831</v>
+        <v>2.124</v>
       </c>
       <c r="E22" t="n">
-        <v>4.831</v>
+        <v>2.196</v>
       </c>
       <c r="F22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
         <v>4</v>
       </c>
-      <c r="G22" t="n">
-        <v>18</v>
-      </c>
-      <c r="H22" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" t="n">
-        <v>3</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
       <c r="K22" t="n">
-        <v>19.3</v>
+        <v>17.6</v>
       </c>
       <c r="L22" t="n">
-        <v>19.3</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Josh Daicos</t>
+          <t>Callum L. Brown</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7421,40 +7480,40 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3.565</v>
+        <v>2.3</v>
       </c>
       <c r="D23" t="n">
-        <v>3.565</v>
+        <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>3.565</v>
+        <v>2.3</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G23" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>17.8</v>
+        <v>16.1</v>
       </c>
       <c r="L23" t="n">
-        <v>17.8</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Will Kelly</t>
+          <t>Jay Rantall</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7463,166 +7522,166 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.822</v>
+        <v>1.203</v>
       </c>
       <c r="D24" t="n">
-        <v>0.638</v>
+        <v>1.203</v>
       </c>
       <c r="E24" t="n">
-        <v>0.822</v>
+        <v>1.203</v>
       </c>
       <c r="F24" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H24" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K24" t="n">
-        <v>16.4</v>
+        <v>15.6</v>
       </c>
       <c r="L24" t="n">
-        <v>16.4</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Callum L. Brown</t>
+          <t>Darcy Cameron</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>utility</t>
+          <t>ruck</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2.3</v>
+        <v>3.567</v>
       </c>
       <c r="D25" t="n">
-        <v>2.3</v>
+        <v>3.567</v>
       </c>
       <c r="E25" t="n">
-        <v>2.3</v>
+        <v>3.567</v>
       </c>
       <c r="F25" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>16.1</v>
+        <v>14.3</v>
       </c>
       <c r="L25" t="n">
-        <v>16.1</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Darcy Cameron</t>
+          <t>Beau McCreery</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ruck</t>
+          <t>pressure_forward</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3.567</v>
+        <v>1.47</v>
       </c>
       <c r="D26" t="n">
-        <v>3.567</v>
+        <v>1.47</v>
       </c>
       <c r="E26" t="n">
-        <v>3.567</v>
+        <v>1.47</v>
       </c>
       <c r="F26" t="n">
+        <v>9</v>
+      </c>
+      <c r="G26" t="n">
+        <v>13</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5</v>
+      </c>
+      <c r="I26" t="n">
         <v>4</v>
       </c>
-      <c r="G26" t="n">
-        <v>18</v>
-      </c>
-      <c r="H26" t="n">
-        <v>4</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
       <c r="J26" t="n">
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>14.3</v>
+        <v>13.2</v>
       </c>
       <c r="L26" t="n">
-        <v>14.3</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Beau McCreery</t>
+          <t>Nathan Murphy</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>pressure_forward</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.47</v>
+        <v>1.855</v>
       </c>
       <c r="D27" t="n">
-        <v>1.47</v>
+        <v>1.855</v>
       </c>
       <c r="E27" t="n">
-        <v>1.47</v>
+        <v>1.855</v>
       </c>
       <c r="F27" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G27" t="n">
+        <v>15</v>
+      </c>
+      <c r="H27" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="L27" t="n">
         <v>13</v>
-      </c>
-      <c r="H27" t="n">
-        <v>5</v>
-      </c>
-      <c r="I27" t="n">
-        <v>4</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="L27" t="n">
-        <v>13.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Nathan Murphy</t>
+          <t>Will Kelly</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7631,34 +7690,34 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.855</v>
+        <v>0.822</v>
       </c>
       <c r="D28" t="n">
-        <v>1.855</v>
+        <v>0.638</v>
       </c>
       <c r="E28" t="n">
-        <v>1.855</v>
+        <v>0.822</v>
       </c>
       <c r="F28" t="n">
+        <v>20</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="n">
+        <v>13</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
         <v>7</v>
       </c>
-      <c r="G28" t="n">
-        <v>15</v>
-      </c>
-      <c r="H28" t="n">
-        <v>5</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
       <c r="K28" t="n">
-        <v>13</v>
+        <v>10.7</v>
       </c>
       <c r="L28" t="n">
-        <v>13</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="29">
@@ -8101,7 +8160,7 @@
         <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>41.4</v>
+        <v>25.8</v>
       </c>
       <c r="E2" t="n">
         <v>41.4</v>
@@ -8110,7 +8169,7 @@
         <v>19.6</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="3">
@@ -8124,7 +8183,7 @@
         <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>39.1</v>
+        <v>25.2</v>
       </c>
       <c r="E3" t="n">
         <v>39.1</v>
@@ -8133,7 +8192,7 @@
         <v>18.1</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -8147,7 +8206,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>38.4</v>
+        <v>24.1</v>
       </c>
       <c r="E4" t="n">
         <v>38.4</v>
@@ -8156,7 +8215,7 @@
         <v>16.5</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="5">
@@ -8170,7 +8229,7 @@
         <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>37.8</v>
+        <v>22.8</v>
       </c>
       <c r="E5" t="n">
         <v>37.8</v>
@@ -8179,7 +8238,7 @@
         <v>16.1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -8193,7 +8252,7 @@
         <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>30.8</v>
       </c>
       <c r="E6" t="n">
         <v>40</v>
@@ -8202,7 +8261,7 @@
         <v>17.9</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -8331,7 +8390,7 @@
         <v>16</v>
       </c>
       <c r="D12" t="n">
-        <v>41.9</v>
+        <v>25.6</v>
       </c>
       <c r="E12" t="n">
         <v>41.9</v>
@@ -8340,7 +8399,7 @@
         <v>19</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="13">
@@ -8354,7 +8413,7 @@
         <v>16</v>
       </c>
       <c r="D13" t="n">
-        <v>46.3</v>
+        <v>32</v>
       </c>
       <c r="E13" t="n">
         <v>46.3</v>
@@ -8363,7 +8422,7 @@
         <v>22.7</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="14">
@@ -8377,7 +8436,7 @@
         <v>16</v>
       </c>
       <c r="D14" t="n">
-        <v>44.4</v>
+        <v>27.9</v>
       </c>
       <c r="E14" t="n">
         <v>44.4</v>
@@ -8386,7 +8445,7 @@
         <v>20.6</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="15">
@@ -8423,7 +8482,7 @@
         <v>16</v>
       </c>
       <c r="D16" t="n">
-        <v>38.8</v>
+        <v>25.6</v>
       </c>
       <c r="E16" t="n">
         <v>38.8</v>
@@ -8432,7 +8491,7 @@
         <v>17.4</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="17">
@@ -8650,7 +8709,7 @@
         <v>177</v>
       </c>
       <c r="D2" t="n">
-        <v>380.4</v>
+        <v>303.9</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -8671,7 +8730,7 @@
         <v>44</v>
       </c>
       <c r="D3" t="n">
-        <v>158</v>
+        <v>145.7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -8692,7 +8751,7 @@
         <v>41</v>
       </c>
       <c r="D4" t="n">
-        <v>145.9</v>
+        <v>140.2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -8713,7 +8772,7 @@
         <v>41</v>
       </c>
       <c r="D5" t="n">
-        <v>125.1</v>
+        <v>104.8</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -8734,7 +8793,7 @@
         <v>28</v>
       </c>
       <c r="D6" t="n">
-        <v>67.90000000000001</v>
+        <v>54.4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -8816,7 +8875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8894,10 +8953,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>injury_weight_pvs</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PVS used for games-missed totals when games played &lt; 14: max(season PVS, last established season).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>pvs_weights</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>See pvs_weights tab. MI50 and intercept marks lift key forwards/defenders toward other roles.</t>
         </is>

</xml_diff>